<commit_message>
v433.0.0: Einzelakten vollständig und layoutgetreu aufbereiten
</commit_message>
<xml_diff>
--- a/testakten/arbeitsrecht-kuendigungsdrama-koerber-werk/14_gehaltsvergleich_koerber_wolters.xlsx
+++ b/testakten/arbeitsrecht-kuendigungsdrama-koerber-werk/14_gehaltsvergleich_koerber_wolters.xlsx
@@ -110,7 +110,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -132,11 +132,55 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -194,6 +238,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -594,6 +640,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
@@ -800,12 +847,21 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
         <is>
           <t>▼  Dr. Annika Körber — Vergleichszeitraum als Werkleiterin Eberswalde (ab 09/2021)</t>
         </is>
       </c>
+      <c r="B11" s="21" t="n"/>
+      <c r="C11" s="21" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="21" t="n"/>
+      <c r="G11" s="21" t="n"/>
+      <c r="H11" s="21" t="n"/>
+      <c r="I11" s="22" t="n"/>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="10" t="n">
@@ -978,12 +1034,19 @@
         <v>-35.7</v>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="32" customHeight="1">
       <c r="A18" s="15" t="inlineStr">
         <is>
           <t>Geschätzte Gesamtdifferenz (Körber-Periode 09/2021–12/2025, annualisiert vs. Wolters-Vergütung)</t>
         </is>
       </c>
+      <c r="B18" s="21" t="n"/>
+      <c r="C18" s="21" t="n"/>
+      <c r="D18" s="21" t="n"/>
+      <c r="E18" s="21" t="n"/>
+      <c r="F18" s="21" t="n"/>
+      <c r="G18" s="22" t="n"/>
       <c r="H18" s="16" t="n">
         <v>-176000</v>
       </c>
@@ -1025,6 +1088,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="19" t="inlineStr">
         <is>
@@ -1045,7 +1109,7 @@
       </c>
       <c r="B4" s="20" t="inlineStr">
         <is>
-          <t>Quelle: mündliche Aussage Cornelia Dratwa (ehemalige Rechnungswesen-Mitarbeiterin, Eberswalde). Bisher keine urkundliche Bestätigung. Beweisantrag auf Vorlage der Vergütungsunterlagen Wolters ist im Klageverfahren vorgesehen (§ 142 ZPO).</t>
+          <t>Quelle: mündliche Aussage Cornelia Dratwa (ehemalige Rechnungswesen-Mitarbeiterin, Eberswalde). Bisher keine urkundliche Bestätigung. Beweisantrag auf Vorlage der Vergütungsunterlagen Wolters ist im Klageverfahren vorgesehen (Paragraf 142 ZPO).</t>
         </is>
       </c>
     </row>
@@ -1093,7 +1157,7 @@
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>§§ 3, 4, 7, 10 EntgTranspG; § 22 AGG; § 3 Abs. 2 MiLoG analog; Art. 157 AEUV. Nachzahlungsanspruch rückwirkend maximal 3 Jahre (§ 195 BGB i.V.m. § 15 Abs. 4 AGG, Fristbeginn frühestens Ende des jeweiligen Jahres).</t>
+          <t>Paragrafen 3, 4, 7, 10 EntgTranspG; Paragraf 22 AGG; Paragraf 3 Abs. 2 MiLoG analog; Art. 157 AEUV. Nachzahlungsanspruch rückwirkend maximal 3 Jahre (Paragraf 195 BGB i.V.m. Paragraf 15 Abs. 4 AGG, Fristbeginn frühestens Ende des jeweiligen Jahres).</t>
         </is>
       </c>
     </row>

</xml_diff>